<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 13:37:49
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -506,44 +506,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>testuser</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{"hash": "9a53317f7f2d82d7271b144573fb777be6ebb3b98e53afdc419136269e29f6f9", "salt": "5433a07dd4678f96d4836ed777751ea90e0fc6dc3fadc4a6409973fdb0f56390", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>test@test.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-07-20T13:37:13.698507</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 14:17:45
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -506,6 +506,44 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>testuser</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "fd91da8db6dd54f7a6cbaa14b13d9792e01579b245daea088f9059b01cb21fe8", "salt": "35c9d57565c53b1fe989c3e60f08ae0234b7e8862ff08c6c422cedd5b116e16f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-20T14:17:45.256067</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 14:17:59
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -506,44 +506,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>testuser</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{"hash": "fd91da8db6dd54f7a6cbaa14b13d9792e01579b245daea088f9059b01cb21fe8", "salt": "35c9d57565c53b1fe989c3e60f08ae0234b7e8862ff08c6c422cedd5b116e16f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>test@test.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-07-20T14:17:45.256067</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[数据同步] 测试创建用户testuser01 - 2026-07-20 16:39:50
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -502,6 +502,44 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>testuser01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "eccf425d66919fa925bbbf2d5a8bd67795c0fc07471b42c1eb37fa87960f124b", "salt": "e49838ddc575a48f01b1083856855cc3f16d895533c108712b260ca1b58b6ef8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:39:39.308702</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 16:48:58
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"hash": "26fa344e8cfcaa47aa136e4272d30a7e18fed6ce5892e3c71f867b2e886d624c", "salt": "92bf9efd33c9f5a547d3448c8672b297f64ea8b8f8525ce479198ac94fe27d53", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "edb65a5eb2621d4e44bed993f7aaba8271aaef0f2ea3f1520a5e688c3e4f0c6e", "salt": "5fcbe93430408b99228183311a4a292305e70a015920d9140abf41cc96732f82", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,7 +487,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-20T10:00:00</t>
+          <t>2026-07-20T16:48:58.174266</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -497,44 +497,6 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>testuser01</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{"hash": "eccf425d66919fa925bbbf2d5a8bd67795c0fc07471b42c1eb37fa87960f124b", "salt": "e49838ddc575a48f01b1083856855cc3f16d895533c108712b260ca1b58b6ef8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>test@test.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-07-20T16:39:39.308702</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 16:52:47
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"hash": "edb65a5eb2621d4e44bed993f7aaba8271aaef0f2ea3f1520a5e688c3e4f0c6e", "salt": "5fcbe93430408b99228183311a4a292305e70a015920d9140abf41cc96732f82", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "26fa344e8cfcaa47aa136e4272d30a7e18fed6ce5892e3c71f867b2e886d624c", "salt": "92bf9efd33c9f5a547d3448c8672b297f64ea8b8f8525ce479198ac94fe27d53", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,7 +487,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-20T16:48:58.174266</t>
+          <t>2026-07-20T10:00:00</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -497,6 +497,82 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>testuser01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "eccf425d66919fa925bbbf2d5a8bd67795c0fc07471b42c1eb37fa87960f124b", "salt": "e49838ddc575a48f01b1083856855cc3f16d895533c108712b260ca1b58b6ef8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:39:39.308702</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>testuser03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"hash": "5853eda22e78b8000515fcf66447336098c8ade5f9232e905f78c8f4bfb64715", "salt": "7a88bb2a034f02cadeb65cb8feb7a920a2b0c713c6d1ef48401abe0fcf7f5d62", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>test03@test.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:52:47.714822</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 16:55:04
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"hash": "c1602efa68ef683851fee5959bac9f72b3890e6260e0945dc503e684bd9a1366", "salt": "cf6a84663bba9780cada09143cf7ac27d96dc6fbb533a358930c84d2eb2669ce", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "23f6cca45a9b218acf6381bba0030e34c2e98457a9e31fca73527136fe767fa3", "salt": "a272d3a901c91b4db241c63c2b1642b6a1f89b5928fc00189de2f033927cd8fb", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -497,6 +497,44 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>test_user1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "bb23529dae8d0d91642d85fafa45a5bf1e9724c49d99d4916da31c9593f55224", "salt": "1003ae75ec187778574ba6ac65532681727172ccab8ff03d832832d405470d21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>test1@test.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:55:04.313343</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 16:55:07
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -540,6 +540,44 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>test_user2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"hash": "b81561b892d3035f6f45e4b7c51f1decfbfb5e07257d8e891ff4941a596a5eb5", "salt": "29eaf52ed75147531c3e3ac6013443d6431bf32d018b22964a55489e20e05508", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>test2@test.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:55:07.071730</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 16:55:12
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,27 +505,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>test_user1</t>
+          <t>test_user2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "bb23529dae8d0d91642d85fafa45a5bf1e9724c49d99d4916da31c9593f55224", "salt": "1003ae75ec187778574ba6ac65532681727172ccab8ff03d832832d405470d21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "b81561b892d3035f6f45e4b7c51f1decfbfb5e07257d8e891ff4941a596a5eb5", "salt": "29eaf52ed75147531c3e3ac6013443d6431bf32d018b22964a55489e20e05508", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>test1@test.com</t>
+          <t>test2@test.com</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T16:55:04.313343</t>
+          <t>2026-07-20T16:55:07.071730</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -535,44 +535,6 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>test_user2</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>{"hash": "b81561b892d3035f6f45e4b7c51f1decfbfb5e07257d8e891ff4941a596a5eb5", "salt": "29eaf52ed75147531c3e3ac6013443d6431bf32d018b22964a55489e20e05508", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>test2@test.com</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-07-20T16:55:07.071730</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 17:32:10
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -502,6 +502,44 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>testuser_e2e</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>test@example.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-20T17:32:10.744283</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 17:32:15
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -540,6 +540,40 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>testuser_push_check</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-20T17:32:15.492701</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 17:38:19
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -574,6 +574,40 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>verify_user_fix</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-07-20T17:38:19.938611</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 17:38:26
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -577,23 +577,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>verify_user_fix</t>
+          <t>verify_push_retry</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:19.938611</t>
+          <t>2026-07-20T17:38:26.953113</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -603,6 +603,40 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>verify_user_fix</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-20T17:38:19.938611</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 17:38:31
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>testuser_e2e</t>
+          <t>e2e_verify_user</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -522,14 +522,10 @@
           <t>editor</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>test@example.com</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T17:32:10.744283</t>
+          <t>2026-07-20T17:38:31.078683</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -547,23 +543,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>testuser_push_check</t>
+          <t>testuser_e2e</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>test@example.com</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T17:32:15.492701</t>
+          <t>2026-07-20T17:32:10.744283</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -581,12 +581,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>verify_push_retry</t>
+          <t>testuser_push_check</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -597,7 +597,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:26.953113</t>
+          <t>2026-07-20T17:32:15.492701</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -615,23 +615,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>verify_user_fix</t>
+          <t>verify_push_retry</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:19.938611</t>
+          <t>2026-07-20T17:38:26.953113</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -641,6 +641,40 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>verify_user_fix</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-07-20T17:38:19.938611</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 17:43:31
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_verify_user</t>
+          <t>e2e_user1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "7b2d637598e5c7ea13d991366e3aadc863db0364aca5986f43304e1538e1accf", "salt": "67ffc55a65de75b72910be9a6e9b7bf98153618e954ace4d3a28b74dcba72fa8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -522,10 +522,14 @@
           <t>editor</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>e2e1@test.com</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:31.078683</t>
+          <t>2026-07-20T17:43:30.999921</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -543,12 +547,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>testuser_e2e</t>
+          <t>e2e_verify_user</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -556,14 +560,10 @@
           <t>editor</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>test@example.com</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T17:32:10.744283</t>
+          <t>2026-07-20T17:38:31.078683</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -581,23 +581,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>testuser_push_check</t>
+          <t>testuser_e2e</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>test@example.com</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T17:32:15.492701</t>
+          <t>2026-07-20T17:32:10.744283</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -615,12 +619,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>verify_push_retry</t>
+          <t>testuser_push_check</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -631,7 +635,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:26.953113</t>
+          <t>2026-07-20T17:32:15.492701</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -649,23 +653,23 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>verify_user_fix</t>
+          <t>verify_push_retry</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:19.938611</t>
+          <t>2026-07-20T17:38:26.953113</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -675,6 +679,40 @@
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>verify_user_fix</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-07-20T17:38:19.938611</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 17:43:33
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -547,23 +547,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_verify_user</t>
+          <t>e2e_user2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9eec3449a220031e4ba232d441784fdc94bc4ccccb91a8a3972a186196fc9e41", "salt": "9009077b42039dad86e9bb866bf04052321d6eb27227bfb934a41c439409311d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>e2e2@test.com</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:31.078683</t>
+          <t>2026-07-20T17:43:33.221399</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -581,12 +585,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>testuser_e2e</t>
+          <t>e2e_verify_user</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -594,14 +598,10 @@
           <t>editor</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>test@example.com</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T17:32:10.744283</t>
+          <t>2026-07-20T17:38:31.078683</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -619,23 +619,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>testuser_push_check</t>
+          <t>testuser_e2e</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>test@example.com</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T17:32:15.492701</t>
+          <t>2026-07-20T17:32:10.744283</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -653,12 +657,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>verify_push_retry</t>
+          <t>testuser_push_check</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -669,7 +673,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:26.953113</t>
+          <t>2026-07-20T17:32:15.492701</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -687,23 +691,23 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>verify_user_fix</t>
+          <t>verify_push_retry</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:19.938611</t>
+          <t>2026-07-20T17:38:26.953113</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -713,6 +717,40 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>verify_user_fix</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-07-20T17:38:19.938611</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 17:43:37
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -509,27 +509,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_user1</t>
+          <t>e2e_user2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "7b2d637598e5c7ea13d991366e3aadc863db0364aca5986f43304e1538e1accf", "salt": "67ffc55a65de75b72910be9a6e9b7bf98153618e954ace4d3a28b74dcba72fa8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9eec3449a220031e4ba232d441784fdc94bc4ccccb91a8a3972a186196fc9e41", "salt": "9009077b42039dad86e9bb866bf04052321d6eb27227bfb934a41c439409311d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>e2e1@test.com</t>
+          <t>e2e2@test.com</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T17:43:30.999921</t>
+          <t>2026-07-20T17:43:33.221399</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -547,27 +547,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_user2</t>
+          <t>e2e_verify_user</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "9eec3449a220031e4ba232d441784fdc94bc4ccccb91a8a3972a186196fc9e41", "salt": "9009077b42039dad86e9bb866bf04052321d6eb27227bfb934a41c439409311d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>e2e2@test.com</t>
-        </is>
-      </c>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T17:43:33.221399</t>
+          <t>2026-07-20T17:38:31.078683</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -585,12 +581,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>e2e_verify_user</t>
+          <t>testuser_e2e</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -598,10 +594,14 @@
           <t>editor</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>test@example.com</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:31.078683</t>
+          <t>2026-07-20T17:32:10.744283</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -619,27 +619,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>testuser_e2e</t>
+          <t>testuser_push_check</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>test@example.com</t>
-        </is>
-      </c>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T17:32:10.744283</t>
+          <t>2026-07-20T17:32:15.492701</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -657,12 +653,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>testuser_push_check</t>
+          <t>verify_push_retry</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -673,7 +669,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T17:32:15.492701</t>
+          <t>2026-07-20T17:38:26.953113</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -691,23 +687,23 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>verify_push_retry</t>
+          <t>verify_user_fix</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:26.953113</t>
+          <t>2026-07-20T17:38:19.938611</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -717,40 +713,6 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>verify_user_fix</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:38:19.938611</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 18:01:09
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -509,27 +509,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_user2</t>
+          <t>e2e_deploy_test</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "9eec3449a220031e4ba232d441784fdc94bc4ccccb91a8a3972a186196fc9e41", "salt": "9009077b42039dad86e9bb866bf04052321d6eb27227bfb934a41c439409311d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d927459d9e7da61f536cd69f6ffdab448113c867ac6b098434c10437c9ec5356", "salt": "9cb9540a5d4c7aaa11057fd3ce43463307e7384a44e5376deb8388972cdb0aa6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>e2e2@test.com</t>
+          <t>e2e@test.com</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T17:43:33.221399</t>
+          <t>2026-07-20T18:01:09.203206</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -547,23 +547,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_verify_user</t>
+          <t>e2e_user2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9eec3449a220031e4ba232d441784fdc94bc4ccccb91a8a3972a186196fc9e41", "salt": "9009077b42039dad86e9bb866bf04052321d6eb27227bfb934a41c439409311d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>e2e2@test.com</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:31.078683</t>
+          <t>2026-07-20T17:43:33.221399</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -581,12 +585,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>testuser_e2e</t>
+          <t>e2e_verify_user</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -594,14 +598,10 @@
           <t>editor</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>test@example.com</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T17:32:10.744283</t>
+          <t>2026-07-20T17:38:31.078683</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -619,23 +619,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>testuser_push_check</t>
+          <t>testuser_e2e</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>test@example.com</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T17:32:15.492701</t>
+          <t>2026-07-20T17:32:10.744283</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -653,12 +657,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>verify_push_retry</t>
+          <t>testuser_push_check</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -669,7 +673,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:26.953113</t>
+          <t>2026-07-20T17:32:15.492701</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -687,23 +691,23 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>verify_user_fix</t>
+          <t>verify_push_retry</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:19.938611</t>
+          <t>2026-07-20T17:38:26.953113</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -713,6 +717,40 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>verify_user_fix</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-07-20T17:38:19.938611</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 18:01:54
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"hash": "58ccb9b289e7d49953ca4808b5f186ffb843b3784657480f6226eb25fe17abf1", "salt": "fe3e83fe502ef8cc4453269c26b48066127cad8ba394f64d45fc595a170b3808", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "a9d1bc3fc07993fa147aecbd5f560af63711ac72c7d223f335fd3791d3823f9c", "salt": "50d5014eea4b55e46e4a7d52b05782ff9ba4afc3f921aaa0fa9edc7e56383a8f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,270 +487,16 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-20T10:00:00</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2099-01-01T00:00:00</t>
-        </is>
-      </c>
+          <t>2026-07-20T18:01:54.642710</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>e2e_deploy_test</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{"hash": "d927459d9e7da61f536cd69f6ffdab448113c867ac6b098434c10437c9ec5356", "salt": "9cb9540a5d4c7aaa11057fd3ce43463307e7384a44e5376deb8388972cdb0aa6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>e2e@test.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-07-20T18:01:09.203206</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>e2e_user2</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>{"hash": "9eec3449a220031e4ba232d441784fdc94bc4ccccb91a8a3972a186196fc9e41", "salt": "9009077b42039dad86e9bb866bf04052321d6eb27227bfb934a41c439409311d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>e2e2@test.com</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:43:33.221399</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>e2e_verify_user</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:38:31.078683</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>testuser_e2e</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>test@example.com</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:32:10.744283</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>testuser_push_check</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:32:15.492701</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>verify_push_retry</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:38:26.953113</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>verify_user_fix</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:38:19.938611</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 18:01:58
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"hash": "a9d1bc3fc07993fa147aecbd5f560af63711ac72c7d223f335fd3791d3823f9c", "salt": "50d5014eea4b55e46e4a7d52b05782ff9ba4afc3f921aaa0fa9edc7e56383a8f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "8f920f413e81d1f005ad6e91c6e1ff977ff1028e669da9797716137382a31e1c", "salt": "82b9f68c7becf9a7914a72610c1cc34bf4d7a49e4cb023657a46011bb2beb956", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,7 +487,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-20T18:01:54.642710</t>
+          <t>2026-07-20T18:01:58.220033</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 18:06:16
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -653,23 +653,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>verify_push_retry</t>
+          <t>verify_fix_user</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "718cc547c96b88e6dc0aab54828318181b3661492013dcffd6fbc7cbc77321e5", "salt": "cd905ef34176cd3dafc276a09690ef3a7c0fc0443b4fa6eb4f852c56376f0241", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>fix@test.com</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:26.953113</t>
+          <t>2026-07-20T18:06:16.032053</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -687,23 +691,23 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>verify_user_fix</t>
+          <t>verify_push_retry</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T17:38:19.938611</t>
+          <t>2026-07-20T17:38:26.953113</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -713,6 +717,40 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>verify_user_fix</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-07-20T17:38:19.938611</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[数据同步] E2E-项目验证，3项变更 - 2026-07-20 18:11:17
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"hash": "58ccb9b289e7d49953ca4808b5f186ffb843b3784657480f6226eb25fe17abf1", "salt": "fe3e83fe502ef8cc4453269c26b48066127cad8ba394f64d45fc595a170b3808", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "97cc8e85c121280137b3802ae2bdfe7c2c609280188fbd1a4c4de5a76c3bae23", "salt": "f4f496d0dc318d49bd49c13ee06483f0bd8f48633b7fc619c051d213510922a3", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -490,267 +490,13 @@
           <t>2026-07-20T10:00:00</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2099-01-01T00:00:00</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>e2e_user2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{"hash": "9eec3449a220031e4ba232d441784fdc94bc4ccccb91a8a3972a186196fc9e41", "salt": "9009077b42039dad86e9bb866bf04052321d6eb27227bfb934a41c439409311d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>e2e2@test.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:43:33.221399</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>e2e_verify_user</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>{"hash": "9a797747f6420265fdb659194a11e909a07e319dddd22af873bd7685c2235361", "salt": "c76bb0c5d38855bd131cbcbb98b9cce186a4c9e463bdcd8dc45edd3e1019bc6f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:38:31.078683</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>testuser_e2e</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>{"hash": "7a9492afd32bcc94fb8f2e4a76082fee516c1118c6fc2eb43a07eb6c4d432105", "salt": "ec27d8b6abee60e73402a6820aea32522023d1d0a4a448964cb27e3eb871be13", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>test@example.com</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:32:10.744283</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>testuser_push_check</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>{"hash": "4fe9894fff48d33bfbd93ac0246b96f389d27cc339dd2e265be7e40810475c15", "salt": "3a433c978fd74991540585641c15b0d9263c0e28f8bbbeedffa5ff5739e3f46b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:32:15.492701</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>verify_fix_user</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>{"hash": "718cc547c96b88e6dc0aab54828318181b3661492013dcffd6fbc7cbc77321e5", "salt": "cd905ef34176cd3dafc276a09690ef3a7c0fc0443b4fa6eb4f852c56376f0241", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>fix@test.com</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-07-20T18:06:16.032053</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>verify_push_retry</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>{"hash": "4ee3416b55fe9aa3bea8ee6bb76fff68ecd506eac9df84179397760b8c852a8f", "salt": "e7238adefaae6ec4d3ccd1ecaa6b7a06cd4121fdacbc4c0761bd112caa638f21", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:38:26.953113</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>verify_user_fix</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>{"hash": "40e7df3f7fec35ef2a6acd568690b5aca4c8e0acf663337fea105c7df8cc9b00", "salt": "a52f59a969f486496339eb4d8a1b7212a02a75da48242a3aa9a6cfa1e08d28ad", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:38:19.938611</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 18:11:23
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"hash": "97cc8e85c121280137b3802ae2bdfe7c2c609280188fbd1a4c4de5a76c3bae23", "salt": "f4f496d0dc318d49bd49c13ee06483f0bd8f48633b7fc619c051d213510922a3", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "bc216350a9b40e83338a39ed55df61e25c079f88c07957d2c5efc7c7a9863dc5", "salt": "443d218fc72b328c85d9cdf7e296cd7a4b4690d661ad84cf9c434f219416eedd", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -497,6 +497,44 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>e2e_account_test</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "e4ffd6058c47f8e29d0da61020fcb7d4195054b38bc7af6c4590da42199c62ac", "salt": "bdc6574861f1bcca61dd978f053f6b19fa45a23e1c671e739c237c461302fc40", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>e2e@test.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-20T18:11:23.467790</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 23:48:39
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -502,6 +502,74 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>persist_test_1243</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:48:39.114271</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>testuser_1243</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:48:39.047971</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-20 23:54:27
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,12 +505,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,7 +521,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -573,12 +573,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>testuser_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.047971</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -599,6 +599,40 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>testuser_1243</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:48:39.047971</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-21 00:20:34
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,12 +505,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>api_test_1470</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "c84ca300c003c85180c52fb255abe60b1398ce3a7373a83f0d9777b95c439b2a", "salt": "689b0a4978431d2c560a9424072a2f006d9cdaeedc937ddf8e1ae3d5b889dfb7", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,7 +521,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-21T00:20:34.436441</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -573,12 +573,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -607,12 +607,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>testuser_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.047971</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -633,6 +633,40 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>testuser_1243</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:48:39.047971</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-21 00:28:47
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>e2e_test_1564</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "81771fba6006a006a1aa6c1117e874104dfb4e2d770801112750e8949ad906a0", "salt": "d3c6222b176bcc35df4d98fb28e2f133d4700dda2aa25d419460626d675cef69", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-21T00:28:47.096326</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -573,12 +573,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -607,12 +607,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -641,12 +641,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>testuser_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -657,7 +657,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.047971</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -667,6 +667,40 @@
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>testuser_1243</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:48:39.047971</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] E2E测试推送 - 2026-07-21 00:30:14
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -573,12 +573,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>e2e_test_1660</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-21T00:30:13.017146</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -607,12 +607,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -641,12 +641,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -657,7 +657,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -675,12 +675,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>testuser_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -691,7 +691,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.047971</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -701,6 +701,40 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>testuser_1243</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:48:39.047971</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 00:33:05
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -607,12 +607,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -641,12 +641,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -657,7 +657,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -675,12 +675,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -691,7 +691,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -709,12 +709,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>testuser_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -725,7 +725,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.047971</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -735,6 +735,40 @@
         </is>
       </c>
       <c r="H9" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>testuser_1243</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:48:39.047971</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:25:53
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="用户表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"hash": "aeef23a0562db11f0f5e9b7153deb85938ab2f9c8f0410b342089c28bae42451", "salt": "acc6a0bb51828ff5b7cef6638b69f6527f1c90b19576090ce469bda497c1a050", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "0790abd126cdabd0146e2b2a0e8140f7703aa003715d351888c3e539a03063df", "salt": "ad94e86cc257a1c2a5476efc33b04dcca31897bc4ddde34c560471a65da4570b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -490,10 +490,14 @@
           <t>2026-07-20T10:00:00</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-07-21T02:25:41.928811</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:26:01
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>api_test_1470</t>
+          <t>e2e_test_1564</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "c84ca300c003c85180c52fb255abe60b1398ce3a7373a83f0d9777b95c439b2a", "salt": "689b0a4978431d2c560a9424072a2f006d9cdaeedc937ddf8e1ae3d5b889dfb7", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "81771fba6006a006a1aa6c1117e874104dfb4e2d770801112750e8949ad906a0", "salt": "d3c6222b176bcc35df4d98fb28e2f133d4700dda2aa25d419460626d675cef69", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:20:34.436441</t>
+          <t>2026-07-21T00:28:47.096326</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -543,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_test_1564</t>
+          <t>e2e_test_1660</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "81771fba6006a006a1aa6c1117e874104dfb4e2d770801112750e8949ad906a0", "salt": "d3c6222b176bcc35df4d98fb28e2f133d4700dda2aa25d419460626d675cef69", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,7 +559,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T00:28:47.096326</t>
+          <t>2026-07-21T00:30:13.017146</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -577,12 +577,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>e2e_test_1660</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -593,7 +593,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T00:30:13.017146</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -627,7 +627,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -645,12 +645,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -661,7 +661,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -679,12 +679,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -695,7 +695,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -713,12 +713,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -729,7 +729,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -739,40 +739,6 @@
         </is>
       </c>
       <c r="H9" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:26:15
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_test_1564</t>
+          <t>e2e_test_1660</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "81771fba6006a006a1aa6c1117e874104dfb4e2d770801112750e8949ad906a0", "salt": "d3c6222b176bcc35df4d98fb28e2f133d4700dda2aa25d419460626d675cef69", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:28:47.096326</t>
+          <t>2026-07-21T00:30:13.017146</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -543,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_test_1660</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,7 +559,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T00:30:13.017146</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -577,12 +577,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -593,7 +593,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -627,7 +627,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -645,12 +645,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -661,7 +661,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -679,12 +679,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -695,7 +695,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -705,40 +705,6 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:26:26
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -608,108 +608,6 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>persist_test_1243</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.114271</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>persist_test_1273</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:53:00.635214</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:27:02
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T02:25:41.928811</t>
+          <t>2026-07-21T02:26:54.987461</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_test_1660</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:30:13.017146</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -543,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,7 +559,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -577,12 +577,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -593,7 +593,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -603,6 +603,74 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>persist_test_1273</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:53:00.635214</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>testuser_1243</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:48:39.047971</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:37:24
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="用户表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -490,7 +490,11 @@
           <t>2026-07-20T10:00:00</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-07-21T02:37:08.858287</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>是</t>
@@ -505,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>api_test_1470</t>
+          <t>e2e_test_1564</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "c84ca300c003c85180c52fb255abe60b1398ce3a7373a83f0d9777b95c439b2a", "salt": "689b0a4978431d2c560a9424072a2f006d9cdaeedc937ddf8e1ae3d5b889dfb7", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "81771fba6006a006a1aa6c1117e874104dfb4e2d770801112750e8949ad906a0", "salt": "d3c6222b176bcc35df4d98fb28e2f133d4700dda2aa25d419460626d675cef69", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,7 +525,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:20:34.436441</t>
+          <t>2026-07-21T00:28:47.096326</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -539,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_test_1564</t>
+          <t>e2e_test_1660</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "81771fba6006a006a1aa6c1117e874104dfb4e2d770801112750e8949ad906a0", "salt": "d3c6222b176bcc35df4d98fb28e2f133d4700dda2aa25d419460626d675cef69", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,7 +559,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T00:28:47.096326</t>
+          <t>2026-07-21T00:30:13.017146</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -573,12 +577,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>e2e_test_1660</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,7 +593,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T00:30:13.017146</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -607,12 +611,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,7 +627,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -641,12 +645,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -657,7 +661,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -675,12 +679,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -691,7 +695,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -709,12 +713,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>test_1236</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -725,7 +729,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-21T02:29:32.086612</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -743,12 +747,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -759,7 +763,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -769,40 +773,6 @@
         </is>
       </c>
       <c r="H10" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:37:44
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"hash": "aeef23a0562db11f0f5e9b7153deb85938ab2f9c8f0410b342089c28bae42451", "salt": "acc6a0bb51828ff5b7cef6638b69f6527f1c90b19576090ce469bda497c1a050", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "f3aec2e00e0c45dea180dd753de3934a2985e8afcec875e345c9f452daaa2bc6", "salt": "9b04900f2c8b36a27f4e3a360c7fc2c45425a6ee5c99a9acbe6a91ea5793f177", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -497,7 +497,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_test_1564</t>
+          <t>e2e_test_1660</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "81771fba6006a006a1aa6c1117e874104dfb4e2d770801112750e8949ad906a0", "salt": "d3c6222b176bcc35df4d98fb28e2f133d4700dda2aa25d419460626d675cef69", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:28:47.096326</t>
+          <t>2026-07-21T00:30:13.017146</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -543,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_test_1660</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,7 +559,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T00:30:13.017146</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -577,12 +577,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -593,7 +593,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -627,7 +627,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -645,12 +645,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -661,7 +661,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -679,12 +679,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>test_1236</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -695,7 +695,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-21T02:29:32.086612</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -713,12 +713,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -729,7 +729,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -739,40 +739,6 @@
         </is>
       </c>
       <c r="H9" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:37:49
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_test_1660</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:30:13.017146</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -543,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,7 +559,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -577,12 +577,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -593,7 +593,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -627,7 +627,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -645,12 +645,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>test_1236</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -661,7 +661,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-21T02:29:32.086612</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -679,12 +679,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -695,7 +695,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -705,40 +705,6 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:37:56
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -543,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,7 +559,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -577,12 +577,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>test_1236</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -593,7 +593,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-21T02:29:32.086612</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -627,7 +627,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -637,74 +637,6 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>test_1236</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-07-21T02:29:32.086612</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:37:59
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -608,40 +608,6 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:38:28
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T02:37:08.858287</t>
+          <t>2026-07-21T02:38:20.905342</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -543,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,7 +559,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -577,12 +577,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -593,7 +593,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -603,6 +603,74 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>persist_test_1273</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:53:00.635214</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>test_1236</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-07-21T02:29:32.086612</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:38:57
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T02:38:20.905342</t>
+          <t>2026-07-21T02:38:49.932106</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -543,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,7 +559,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -569,108 +569,6 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>persist_test_1243</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.114271</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>persist_test_1273</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:53:00.635214</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>test_1236</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-07-21T02:29:32.086612</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:39:04
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -540,40 +540,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>persist_test_1273</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:53:00.635214</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:39:09
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -506,40 +506,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>persist_test_1243</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.114271</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:39:37
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T02:38:49.932106</t>
+          <t>2026-07-21T02:39:29.986670</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,6 +501,40 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>persist_test_1273</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:53:00.635214</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:39:41
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -506,40 +506,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>persist_test_1273</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:53:00.635214</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:40:10
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T02:39:29.986670</t>
+          <t>2026-07-21T02:39:56.575410</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,6 +501,40 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>xjq</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "3abe2d7ad3cf93465e8e9c779db6f0586b18fcd219ac381e35f74fa6f7f876ec", "salt": "f060e013066e2c17d62d42056da5793ca65cdf78f6ab40cd58ae2924aa9130f7", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-21T02:40:10.276728</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:41:48
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T02:39:56.575410</t>
+          <t>2026-07-21T02:41:24.830002</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -535,6 +535,40 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>yzz</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"hash": "b099582e66e0c6c576cc6ac7900dcab8eafae9c919ea814f3cc8314266935640", "salt": "dc30d0c28b979a1528072a2a729394fd86545b222cb9fa171b1f2ac04f78a3b3", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-21T02:41:48.221464</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 02:42:04
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -543,12 +543,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "b099582e66e0c6c576cc6ac7900dcab8eafae9c919ea814f3cc8314266935640", "salt": "dc30d0c28b979a1528072a2a729394fd86545b222cb9fa171b1f2ac04f78a3b3", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "b390865c0cc332751288e1c03d415d4dba86323ccc3640bea319f43071b57791", "salt": "74db69a6c45f6d1414caf51a7e8efb4c53bbbadaf5d2ffea92aae9af17ef462c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,7 +559,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T02:41:48.221464</t>
+          <t>2026-07-21T02:42:04.626733</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -569,6 +569,40 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>yzz</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>{"hash": "b099582e66e0c6c576cc6ac7900dcab8eafae9c919ea814f3cc8314266935640", "salt": "dc30d0c28b979a1528072a2a729394fd86545b222cb9fa171b1f2ac04f78a3b3", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-07-21T02:41:48.221464</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 用户admin增量同步，1项变更 - 2026-07-21 02:58:53
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T02:41:24.830002</t>
+          <t>2026-07-21T02:57:32.969990</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -528,7 +528,11 @@
           <t>2026-07-21T02:40:10.276728</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-07-21T02:57:51.469942</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>否</t>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:07:02
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="用户表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"hash": "5a5b7d2de1fe901852df8c6be2cc9c4ea42abf9af6f6f3a0b0bc6cfda8606ee5", "salt": "d99b75b548b204af996c478fa491eb13d666a60e7e352d5adbc91cef1376c7eb", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "aeef23a0562db11f0f5e9b7153deb85938ab2f9c8f0410b342089c28bae42451", "salt": "acc6a0bb51828ff5b7cef6638b69f6527f1c90b19576090ce469bda497c1a050", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -490,14 +490,10 @@
           <t>2026-07-20T10:00:00</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-07-21T02:57:32.969990</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -509,30 +505,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>e2e_test_1564</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "3abe2d7ad3cf93465e8e9c779db6f0586b18fcd219ac381e35f74fa6f7f876ec", "salt": "f060e013066e2c17d62d42056da5793ca65cdf78f6ab40cd58ae2924aa9130f7", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "81771fba6006a006a1aa6c1117e874104dfb4e2d770801112750e8949ad906a0", "salt": "d3c6222b176bcc35df4d98fb28e2f133d4700dda2aa25d419460626d675cef69", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T02:40:10.276728</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-07-21T02:57:51.469942</t>
-        </is>
-      </c>
+          <t>2026-07-21T00:28:47.096326</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>否</t>
@@ -547,23 +539,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>e2e_test_1660</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "b390865c0cc332751288e1c03d415d4dba86323ccc3640bea319f43071b57791", "salt": "74db69a6c45f6d1414caf51a7e8efb4c53bbbadaf5d2ffea92aae9af17ef462c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T02:42:04.626733</t>
+          <t>2026-07-21T00:30:13.017146</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -581,23 +573,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "b099582e66e0c6c576cc6ac7900dcab8eafae9c919ea814f3cc8314266935640", "salt": "dc30d0c28b979a1528072a2a729394fd86545b222cb9fa171b1f2ac04f78a3b3", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T02:41:48.221464</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -607,6 +599,176 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>fix_test_1344</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:54:27.066760</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>persist_test_1243</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:48:39.114271</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>persist_test_1273</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:53:00.635214</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>test_1236</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-07-21T02:29:32.086612</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>testuser_1243</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-07-20T23:48:39.047971</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:07:17
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,12 +505,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_test_1564</t>
+          <t>e2e_test_1660</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "81771fba6006a006a1aa6c1117e874104dfb4e2d770801112750e8949ad906a0", "salt": "d3c6222b176bcc35df4d98fb28e2f133d4700dda2aa25d419460626d675cef69", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,7 +521,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:28:47.096326</t>
+          <t>2026-07-21T00:30:13.017146</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_test_1660</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T00:30:13.017146</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -573,12 +573,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -607,12 +607,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -641,12 +641,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -657,7 +657,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -675,12 +675,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>test_1236</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -691,7 +691,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-21T02:29:32.086612</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -709,12 +709,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -725,7 +725,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -735,40 +735,6 @@
         </is>
       </c>
       <c r="H9" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:07:32
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,12 +505,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_test_1660</t>
+          <t>e2e_test_1749</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "e2869474a10965c8c973f8dc58703f8054899ca7d41a3fd1cd6a4921664cfb0a", "salt": "e1fa1e601e23d0e6a5fb2b0bf48d91e35282f04bb01a8440b10d9f21dd539ddf", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,7 +521,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:30:13.017146</t>
+          <t>2026-07-21T00:33:04.112194</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -573,12 +573,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -607,12 +607,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -641,12 +641,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>test_1236</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -657,7 +657,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-21T02:29:32.086612</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -675,12 +675,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -691,7 +691,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -701,40 +701,6 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:07:44
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,12 +505,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e2e_test_1749</t>
+          <t>fix_test_1344</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "36f0e6d87a5b582e83e49c952981c5e00eb7ad1be1bf45d15ab5c6196a4a9227", "salt": "6da79db6234e757ddac69d3b6b347d5775fb2d62c6e110fb55af7aabad88942d", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,7 +521,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T00:33:04.112194</t>
+          <t>2026-07-20T23:54:27.066760</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -573,12 +573,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -607,12 +607,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>test_1236</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-21T02:29:32.086612</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -641,12 +641,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -657,7 +657,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -667,40 +667,6 @@
         </is>
       </c>
       <c r="H7" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:07:57
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,12 +505,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fix_test_1344</t>
+          <t>persist_test_1243</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "6b7fa9401d012ed9625b52b400410b02defb6fd9e20293a7af9f9ae7bb4278a1", "salt": "46b5a4b166960960517419d837e5b1d7d62c0ef8a8a36a5b6b39e0a94d12534c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,7 +521,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T23:54:27.066760</t>
+          <t>2026-07-20T23:48:39.114271</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -573,12 +573,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>test_1236</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-21T02:29:32.086612</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -607,12 +607,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -633,40 +633,6 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:08:12
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,12 +505,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>persist_test_1243</t>
+          <t>persist_test_1273</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "2417b463e4a1c95541b78586569f9f623f2b86898f56383adf64e5056f21e844", "salt": "e3f743d12640815360bf0203bd182d32ae6a30f6a7d6007acfc3c0bbac1b190b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,7 +521,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T23:48:39.114271</t>
+          <t>2026-07-20T23:53:00.635214</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>test_1236</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-21T02:29:32.086612</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -573,12 +573,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -599,40 +599,6 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:08:26
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,12 +505,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>persist_test_1273</t>
+          <t>test_1236</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "5fc37f0857a1cf7af68606b70c2b18bf038855a8bfe8ab1425177454e4e4aa5a", "salt": "6d0c0e5371420a7823a6d48f3652e15ede787d92da68d0e3691d74490dd25b3c", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,7 +521,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-20T23:53:00.635214</t>
+          <t>2026-07-21T02:29:32.086612</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -565,40 +565,6 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:08:40
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,12 +505,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>test_1236</t>
+          <t>testuser_1243</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "d1de44096be69c38578ccdfe83219a53386cf842ffe954257d9e27a92c4e704c", "salt": "2ea8c875c7c1f7cc51a027268010f9f48b8c16279516b1c9528fbbd56c9e1057", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,7 +521,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T02:29:32.086612</t>
+          <t>2026-07-20T23:48:39.047971</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -531,40 +531,6 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:08:54
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -502,40 +502,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>testuser_1243</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{"hash": "751662d925f083299a9ea47b0ad99754500e635b0e2a1a0af6252a2d69eab5e0", "salt": "1a67ff4459dc4a873937d1f35fae7fb16f04593f14c40038e1277154c8e06d29", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-07-20T23:48:39.047971</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:45:41
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="用户表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T03:14:26.548234</t>
+          <t>2026-07-21T03:44:57.937898</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,6 +501,40 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>xjq</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "404d2f0fe7a6df1a3e79428a8f5f44ad9964ea2ff369b6f7040f5fc7c2b910d1", "salt": "803af3332360107e6ebc39c85c238db440239929747e0c09e5decfc98e9c3112", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-21T03:45:41.134054</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:47:48
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -528,13 +528,51 @@
           <t>2026-07-21T03:45:41.134054</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-07-21T03:47:11.699308</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>yzz</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"hash": "74814fbbeeb4f546cffd11c1598ff89d21bcf4e94aa730bb5b63b3dee0d88c2b", "salt": "4161c60ab4d25dc7ce2099c17ed69c12acb93a4760f3bf25ac865e1577ea26c8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-21T03:47:47.701534</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:48:04
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -547,12 +547,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "74814fbbeeb4f546cffd11c1598ff89d21bcf4e94aa730bb5b63b3dee0d88c2b", "salt": "4161c60ab4d25dc7ce2099c17ed69c12acb93a4760f3bf25ac865e1577ea26c8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "207cddfc59ce077501e611965657d4ba727b39721b05b75f7d30672b997fddb9", "salt": "f36af667fc59b6c3a6f9bbcec36dce6d65b7071d76291070a1739309b3f3ddf4", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -563,7 +563,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T03:47:47.701534</t>
+          <t>2026-07-21T03:48:04.308710</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -573,6 +573,40 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>yzz</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>{"hash": "74814fbbeeb4f546cffd11c1598ff89d21bcf4e94aa730bb5b63b3dee0d88c2b", "salt": "4161c60ab4d25dc7ce2099c17ed69c12acb93a4760f3bf25ac865e1577ea26c8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-07-21T03:47:47.701534</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:48:20
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -509,30 +509,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>flora</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "404d2f0fe7a6df1a3e79428a8f5f44ad9964ea2ff369b6f7040f5fc7c2b910d1", "salt": "803af3332360107e6ebc39c85c238db440239929747e0c09e5decfc98e9c3112", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5a5beb0e56a7a1ce18f639b97d0b690d53dd899c5bb8fdff1df3b225f0ba72f0", "salt": "1f3ef3ff2b2b4c38643d03befcb861a80fd3f6ba579a1bd12f895205e5074149", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T03:45:41.134054</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-07-21T03:47:11.699308</t>
-        </is>
-      </c>
+          <t>2026-07-21T03:48:19.811266</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>否</t>
@@ -547,26 +543,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "207cddfc59ce077501e611965657d4ba727b39721b05b75f7d30672b997fddb9", "salt": "f36af667fc59b6c3a6f9bbcec36dce6d65b7071d76291070a1739309b3f3ddf4", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "404d2f0fe7a6df1a3e79428a8f5f44ad9964ea2ff369b6f7040f5fc7c2b910d1", "salt": "803af3332360107e6ebc39c85c238db440239929747e0c09e5decfc98e9c3112", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T03:48:04.308710</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>2026-07-21T03:45:41.134054</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-07-21T03:47:11.699308</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>否</t>
@@ -581,12 +581,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "74814fbbeeb4f546cffd11c1598ff89d21bcf4e94aa730bb5b63b3dee0d88c2b", "salt": "4161c60ab4d25dc7ce2099c17ed69c12acb93a4760f3bf25ac865e1577ea26c8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "207cddfc59ce077501e611965657d4ba727b39721b05b75f7d30672b997fddb9", "salt": "f36af667fc59b6c3a6f9bbcec36dce6d65b7071d76291070a1739309b3f3ddf4", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -597,7 +597,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T03:47:47.701534</t>
+          <t>2026-07-21T03:48:04.308710</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -607,6 +607,40 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>yzz</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>{"hash": "74814fbbeeb4f546cffd11c1598ff89d21bcf4e94aa730bb5b63b3dee0d88c2b", "salt": "4161c60ab4d25dc7ce2099c17ed69c12acb93a4760f3bf25ac865e1577ea26c8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-21T03:47:47.701534</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 03:49:24
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T03:44:57.937898</t>
+          <t>2026-07-21T03:49:01.544842</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -543,30 +543,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>lhl</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "404d2f0fe7a6df1a3e79428a8f5f44ad9964ea2ff369b6f7040f5fc7c2b910d1", "salt": "803af3332360107e6ebc39c85c238db440239929747e0c09e5decfc98e9c3112", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "4793989a3e2d986efcb19925f19acbae18ba520c43101608a0a1b00368ee7a24", "salt": "fa4c1f3885432e4599545d2b84f8b08a15cc26ae9c16857b2a5d55587d503e52", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T03:45:41.134054</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-07-21T03:47:11.699308</t>
-        </is>
-      </c>
+          <t>2026-07-21T03:49:24.238158</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>否</t>
@@ -581,26 +577,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "207cddfc59ce077501e611965657d4ba727b39721b05b75f7d30672b997fddb9", "salt": "f36af667fc59b6c3a6f9bbcec36dce6d65b7071d76291070a1739309b3f3ddf4", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "404d2f0fe7a6df1a3e79428a8f5f44ad9964ea2ff369b6f7040f5fc7c2b910d1", "salt": "803af3332360107e6ebc39c85c238db440239929747e0c09e5decfc98e9c3112", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T03:48:04.308710</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>2026-07-21T03:45:41.134054</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-07-21T03:47:11.699308</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>否</t>
@@ -615,12 +615,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "74814fbbeeb4f546cffd11c1598ff89d21bcf4e94aa730bb5b63b3dee0d88c2b", "salt": "4161c60ab4d25dc7ce2099c17ed69c12acb93a4760f3bf25ac865e1577ea26c8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "207cddfc59ce077501e611965657d4ba727b39721b05b75f7d30672b997fddb9", "salt": "f36af667fc59b6c3a6f9bbcec36dce6d65b7071d76291070a1739309b3f3ddf4", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -631,7 +631,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-21T03:47:47.701534</t>
+          <t>2026-07-21T03:48:04.308710</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -641,6 +641,40 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>yzz</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>{"hash": "74814fbbeeb4f546cffd11c1598ff89d21bcf4e94aa730bb5b63b3dee0d88c2b", "salt": "4161c60ab4d25dc7ce2099c17ed69c12acb93a4760f3bf25ac865e1577ea26c8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-07-21T03:47:47.701534</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 测试新增项目，1项变更 - 2026-07-21 04:23:47
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="用户表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T03:49:01.544842</t>
+          <t>2026-07-21T03:14:26.548234</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,180 +501,6 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>flora</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{"hash": "5a5beb0e56a7a1ce18f639b97d0b690d53dd899c5bb8fdff1df3b225f0ba72f0", "salt": "1f3ef3ff2b2b4c38643d03befcb861a80fd3f6ba579a1bd12f895205e5074149", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-07-21T03:48:19.811266</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>lhl</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>{"hash": "4793989a3e2d986efcb19925f19acbae18ba520c43101608a0a1b00368ee7a24", "salt": "fa4c1f3885432e4599545d2b84f8b08a15cc26ae9c16857b2a5d55587d503e52", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-07-21T03:49:24.238158</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>xjq</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>{"hash": "404d2f0fe7a6df1a3e79428a8f5f44ad9964ea2ff369b6f7040f5fc7c2b910d1", "salt": "803af3332360107e6ebc39c85c238db440239929747e0c09e5decfc98e9c3112", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-07-21T03:45:41.134054</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-07-21T03:47:11.699308</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ycx</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>{"hash": "207cddfc59ce077501e611965657d4ba727b39721b05b75f7d30672b997fddb9", "salt": "f36af667fc59b6c3a6f9bbcec36dce6d65b7071d76291070a1739309b3f3ddf4", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-07-21T03:48:04.308710</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>yzz</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>{"hash": "74814fbbeeb4f546cffd11c1598ff89d21bcf4e94aa730bb5b63b3dee0d88c2b", "salt": "4161c60ab4d25dc7ce2099c17ed69c12acb93a4760f3bf25ac865e1577ea26c8", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>editor</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-07-21T03:47:47.701534</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[用户同步] 更新用户数据 - 2026-07-21 04:29:08
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -506,6 +506,40 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>xjq</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"hash": "b3ede61899a8b1edb7da0352137d8d8574cecd905ffb1b3aa00432795a473e54", "salt": "79756621ced4fa7d8f73975f1b9ccf48ad9a2ff9a34b8240ef092ce9f66e552e", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-21T04:29:08.529075</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[API同步] 用户admin增量同步，1项变更 - 2026-07-21 05:06:00
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="用户表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T03:14:26.548234</t>
+          <t>2026-07-21T05:05:01.055913</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -530,7 +530,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-21T04:31:51.233766</t>
+          <t>2026-07-21T05:04:42.752463</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 用户xjq增量同步，2项变更 - 2026-07-21 05:12:42
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="用户表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -530,7 +530,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-21T05:09:14.578007</t>
+          <t>2026-07-21T05:12:39.151844</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] admin删除项目 - 2026-07-21 09:07:26
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="用户表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T05:36:44.755654</t>
+          <t>2026-07-21T09:06:55.861985</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq删除项目 - 2026-07-21 10:23:09
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T10:22:14.804654</t>
+          <t>2026-07-21T10:18:00.479077</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-21T10:20:15.573935</t>
+          <t>2026-07-21T10:22:51.643793</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 测试推送 - 2026-07-21 10:48:26
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="用户表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T10:24:59.378572</t>
+          <t>2026-07-21T05:36:44.755654</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-21T10:22:51.643793</t>
+          <t>2026-07-21T05:19:25.360912</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] admin删除项目 - 2026-07-21 11:22:38
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="用户表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T05:36:44.755654</t>
+          <t>2026-07-21T11:22:15.997811</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 用户admin增量同步，重试推送 - 2026-07-21 14:26:21
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T13:56:11.116704</t>
+          <t>2026-07-21T14:22:57.297468</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-21T14:19:33.957341</t>
+          <t>2026-07-21T14:25:46.100711</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-21 14:29:59
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -649,12 +649,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -665,7 +665,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
+          <t>2026-07-21T14:29:59.201564</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -675,6 +675,40 @@
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>yzz</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 用户yjl增量同步，重试推送 - 2026-07-21 14:50:49
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-21T14:22:57.297468</t>
+          <t>2026-07-21T14:31:19.398556</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -668,7 +668,11 @@
           <t>2026-07-21T14:29:59.201564</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-07-21T14:49:44.806631</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>否</t>

</xml_diff>

<commit_message>
[API同步] 用户xjq增量同步，重试推送 - 2026-07-22 07:43:03
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-21T14:25:46.100711</t>
+          <t>2026-07-22T07:42:46.024617</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-21T14:49:44.806631</t>
+          <t>2026-07-22T07:40:11.926249</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-23 00:58:23
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -598,7 +598,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-22T09:22:47.880924</t>
+          <t>2026-07-23T00:57:51.760203</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -713,6 +713,40 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>{"hash": "d7fbd1e86fa4497da2e09be076acddd5dfe610e4ebe176e281542567a9b0bd18", "salt": "291d2a379e9b349f1daf48eb0c6aff61a2dd3b01a946f407016e9042fb808e20", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>editor</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-07-23T00:58:22.865573</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-23 04:38:34
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-23T02:48:06.259686</t>
+          <t>2026-07-23T04:38:08.429606</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -726,12 +726,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "d7fbd1e86fa4497da2e09be076acddd5dfe610e4ebe176e281542567a9b0bd18", "salt": "291d2a379e9b349f1daf48eb0c6aff61a2dd3b01a946f407016e9042fb808e20", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>

</xml_diff>

<commit_message>
[API同步] yzz编辑项目 - 2026-07-23 05:43:41
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-23T04:38:08.429606</t>
+          <t>2026-07-23T05:39:33.816871</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -706,7 +706,11 @@
           <t>2026-07-21T05:24:08.554209</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>否</t>
@@ -740,7 +744,11 @@
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:42:22.818595</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>否</t>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-23 05:45:43
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -577,30 +577,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>lhl</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "f8f8de6fab17c4156f58d63b8032586f5475107dd455afb48f34c51ec5863671", "salt": "87e67563dcab6b352e8fb4ae69ea09406ee6ab46bf53767a96d80627edf6f1e0", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T04:29:08.529075</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-07-23T05:39:33.816871</t>
-        </is>
-      </c>
+          <t>2026-07-23T05:45:42.431806</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>否</t>
@@ -615,26 +611,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:24.754665</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>2026-07-21T04:29:08.529075</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:45:04.719637</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>否</t>
@@ -649,12 +649,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>yjl</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -665,14 +665,10 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-21T14:29:59.201564</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2026-07-22T07:45:30.020648</t>
-        </is>
-      </c>
+          <t>2026-07-21T05:24:24.754665</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>否</t>
@@ -687,12 +683,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -703,12 +699,12 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
+          <t>2026-07-21T14:29:59.201564</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-23T05:43:14.630942</t>
+          <t>2026-07-22T07:45:30.020648</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -725,36 +721,74 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>2026-07-23T05:42:22.818595</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] xjq归档项目 - 2026-07-23 05:49:21
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -596,7 +596,11 @@
           <t>2026-07-23T05:45:42.431806</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:47:54.833218</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>否</t>
@@ -632,7 +636,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-23T05:45:04.719637</t>
+          <t>2026-07-23T05:48:43.927026</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -780,7 +784,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-23T05:42:22.818595</t>
+          <t>2026-07-23T05:46:40.725622</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq批量导入14个项目 - 2026-07-23 05:56:06
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-23T05:47:54.833218</t>
+          <t>2026-07-23T05:53:49.621711</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-23T05:48:43.927026</t>
+          <t>2026-07-23T05:54:56.731343</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq归档项目 - 2026-07-23 06:28:20
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-23T05:53:49.621711</t>
+          <t>2026-07-23T06:26:53.941671</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-23T05:54:56.731343</t>
+          <t>2026-07-23T06:28:00.232968</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-23T05:46:40.725622</t>
+          <t>2026-07-23T06:27:36.743690</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-23 07:16:35
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -615,30 +615,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>tjs</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "ff481015559bcbcaf62f8a10eb4476b76b9a48030e189473eae593876bc87d59", "salt": "e95f6a23a1483d8bdc1dfc159589dd1a1232bb5529eb7da8c629950f6aa68f46", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-21T04:29:08.529075</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026-07-23T07:12:38.408253</t>
-        </is>
-      </c>
+          <t>2026-07-23T07:16:34.409165</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>否</t>
@@ -653,26 +649,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:24.754665</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>2026-07-21T04:29:08.529075</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-07-23T07:12:38.408253</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>否</t>
@@ -687,12 +687,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>yjl</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -703,14 +703,10 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-21T14:29:59.201564</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2026-07-22T07:45:30.020648</t>
-        </is>
-      </c>
+          <t>2026-07-21T05:24:24.754665</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>否</t>
@@ -725,12 +721,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -741,12 +737,12 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
+          <t>2026-07-21T14:29:59.201564</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-23T05:43:14.630942</t>
+          <t>2026-07-22T07:45:30.020648</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -763,36 +759,74 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>2026-07-23T06:27:36.743690</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] tjs新增项目: 非洲工装-曾翔 - 2026-07-23 07:21:11
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -634,7 +634,11 @@
           <t>2026-07-23T07:16:34.409165</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-07-23T07:19:47.613466</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>否</t>

</xml_diff>

<commit_message>
[API同步] xjq归档项目 - 2026-07-23 08:20:35
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -615,28 +615,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tjs</t>
+          <t>mwh</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "ff481015559bcbcaf62f8a10eb4476b76b9a48030e189473eae593876bc87d59", "salt": "e95f6a23a1483d8bdc1dfc159589dd1a1232bb5529eb7da8c629950f6aa68f46", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "04849fccab8734257b614a7f3606554f8caeba646c486aa184611893df552b60", "salt": "ecd2366a8275ec9f74a4608b7f239ed77288c66e565865577cd6b899ea48ec90", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-23T07:16:34.409165</t>
+          <t>2026-07-23T07:28:50.402064</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-23T07:19:47.613466</t>
+          <t>2026-07-23T08:17:45.512455</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -653,28 +653,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>tjs</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "ff481015559bcbcaf62f8a10eb4476b76b9a48030e189473eae593876bc87d59", "salt": "e95f6a23a1483d8bdc1dfc159589dd1a1232bb5529eb7da8c629950f6aa68f46", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-21T04:29:08.529075</t>
+          <t>2026-07-23T07:16:34.409165</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-23T07:12:38.408253</t>
+          <t>2026-07-23T07:19:47.613466</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -691,26 +691,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:24.754665</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>2026-07-21T04:29:08.529075</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-07-23T08:18:21.707906</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>否</t>
@@ -725,12 +729,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>yjl</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -741,14 +745,10 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-21T14:29:59.201564</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2026-07-22T07:45:30.020648</t>
-        </is>
-      </c>
+          <t>2026-07-21T05:24:24.754665</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>否</t>
@@ -763,12 +763,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -779,12 +779,12 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
+          <t>2026-07-21T14:29:59.201564</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-23T05:43:14.630942</t>
+          <t>2026-07-22T07:45:30.020648</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -801,36 +801,74 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>2026-07-23T06:27:36.743690</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] xjq编辑项目 - 2026-07-23 09:05:20
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -636,7 +636,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-23T08:17:45.512455</t>
+          <t>2026-07-23T09:03:42.507286</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-23T08:18:21.707906</t>
+          <t>2026-07-23T09:05:00.395286</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq编辑项目 - 2026-07-23 09:06:59
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -636,7 +636,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-23T09:03:42.507286</t>
+          <t>2026-07-23T09:05:45.102709</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-23T09:05:00.395286</t>
+          <t>2026-07-23T09:06:34.707665</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq编辑项目 - 2026-07-23 09:35:59
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -636,7 +636,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-23T09:09:26.669390</t>
+          <t>2026-07-23T09:31:15.091537</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-23T09:20:02.082020</t>
+          <t>2026-07-23T09:33:36.193097</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq拒绝审批ROW-50 - 2026-07-23 10:52:47
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -636,7 +636,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-23T10:43:54.010513</t>
+          <t>2026-07-23T10:51:12.555060</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-23T10:42:11.398574</t>
+          <t>2026-07-23T10:52:17.853571</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] tjs新增项目: 研究院LoRaWAN - 2026-07-24 05:54:07
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-23T06:26:53.941671</t>
+          <t>2026-07-24T02:47:09.177183</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-23T07:19:47.613466</t>
+          <t>2026-07-24T05:51:30.972507</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-23T06:27:36.743690</t>
+          <t>2026-07-24T05:21:32.385809</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-24 07:40:43
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -543,23 +543,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>flora</t>
+          <t>dajinyu</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "5fc51a63f31c86fafce838506de34c1a4822c35e4eb96313622bb3bb12ddb27a", "salt": "046da8c3e3793dc75e716aca13e50e008d0489f7bf9f7dd8e57f0f4b3420154f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "bf8f6de799a7eed9960cc632206baf3714cb8ff2c80be5ed9b4da42cb43f1479", "salt": "7912bbead6671352fdc02410d7dde4006511e2a25d395403478fe021eb682307", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-21T05:26:59.748591</t>
+          <t>2026-07-24T07:40:42.773933</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -577,30 +577,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>lhl</t>
+          <t>flora</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "f8f8de6fab17c4156f58d63b8032586f5475107dd455afb48f34c51ec5863671", "salt": "87e67563dcab6b352e8fb4ae69ea09406ee6ab46bf53767a96d80627edf6f1e0", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc51a63f31c86fafce838506de34c1a4822c35e4eb96313622bb3bb12ddb27a", "salt": "046da8c3e3793dc75e716aca13e50e008d0489f7bf9f7dd8e57f0f4b3420154f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-23T05:45:42.431806</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-07-24T02:47:09.177183</t>
-        </is>
-      </c>
+          <t>2026-07-21T05:26:59.748591</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>否</t>
@@ -615,12 +611,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>mwh</t>
+          <t>lhl</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "04849fccab8734257b614a7f3606554f8caeba646c486aa184611893df552b60", "salt": "ecd2366a8275ec9f74a4608b7f239ed77288c66e565865577cd6b899ea48ec90", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "f8f8de6fab17c4156f58d63b8032586f5475107dd455afb48f34c51ec5863671", "salt": "87e67563dcab6b352e8fb4ae69ea09406ee6ab46bf53767a96d80627edf6f1e0", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -631,12 +627,12 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-23T07:28:50.402064</t>
+          <t>2026-07-23T05:45:42.431806</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-23T11:12:36.939226</t>
+          <t>2026-07-24T02:47:09.177183</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -653,28 +649,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tjs</t>
+          <t>mwh</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "ff481015559bcbcaf62f8a10eb4476b76b9a48030e189473eae593876bc87d59", "salt": "e95f6a23a1483d8bdc1dfc159589dd1a1232bb5529eb7da8c629950f6aa68f46", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "04849fccab8734257b614a7f3606554f8caeba646c486aa184611893df552b60", "salt": "ecd2366a8275ec9f74a4608b7f239ed77288c66e565865577cd6b899ea48ec90", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-23T07:16:34.409165</t>
+          <t>2026-07-23T07:28:50.402064</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-24T05:51:30.972507</t>
+          <t>2026-07-23T11:12:36.939226</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -691,28 +687,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>tjs</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "ff481015559bcbcaf62f8a10eb4476b76b9a48030e189473eae593876bc87d59", "salt": "e95f6a23a1483d8bdc1dfc159589dd1a1232bb5529eb7da8c629950f6aa68f46", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-21T04:29:08.529075</t>
+          <t>2026-07-23T07:16:34.409165</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-24T05:55:59.574010</t>
+          <t>2026-07-24T05:51:30.972507</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -729,26 +725,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:24.754665</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>2026-07-21T04:29:08.529075</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-07-24T05:55:59.574010</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>否</t>
@@ -763,12 +763,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>yjl</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -779,14 +779,10 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-21T14:29:59.201564</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-07-22T07:45:30.020648</t>
-        </is>
-      </c>
+          <t>2026-07-21T05:24:24.754665</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>否</t>
@@ -801,12 +797,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -817,12 +813,12 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
+          <t>2026-07-21T14:29:59.201564</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-23T05:43:14.630942</t>
+          <t>2026-07-22T07:45:30.020648</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -839,36 +835,74 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>2026-07-24T05:21:32.385809</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 用户ycx增量同步，重试推送 - 2026-07-24 08:11:02
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -782,7 +782,11 @@
           <t>2026-07-21T05:24:24.754665</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-07-24T08:08:35.784199</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>否</t>

</xml_diff>

<commit_message>
[API同步] xjq归档项目 - 2026-07-24 12:46:06
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -562,7 +562,11 @@
           <t>2026-07-24T07:40:42.773933</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-07-24T12:42:40.776957</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>否</t>
@@ -746,7 +750,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-24T05:55:59.574010</t>
+          <t>2026-07-24T12:45:46.871966</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-27 00:22:57
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -767,30 +767,26 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq-cs</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:24.754665</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-07-24T08:08:35.784199</t>
-        </is>
-      </c>
+          <t>2026-07-27T00:22:56.634377</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>否</t>
@@ -805,12 +801,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>yjl</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -821,12 +817,12 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-21T14:29:59.201564</t>
+          <t>2026-07-21T05:24:24.754665</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-22T07:45:30.020648</t>
+          <t>2026-07-24T08:08:35.784199</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -843,12 +839,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -859,12 +855,12 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
+          <t>2026-07-21T14:29:59.201564</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-23T05:43:14.630942</t>
+          <t>2026-07-22T07:45:30.020648</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -881,36 +877,74 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>2026-07-24T05:21:32.385809</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] xjq新增项目: 测试看板 - 2026-07-27 00:25:09
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -750,7 +750,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-27T00:08:33.730248</t>
+          <t>2026-07-27T00:23:17.937689</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -786,7 +786,11 @@
           <t>2026-07-27T00:22:56.634377</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-07-27T00:23:32.727849</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>否</t>

</xml_diff>

<commit_message>
[API同步] xjq归档项目 - 2026-07-27 06:05:38
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-24T12:42:40.776957</t>
+          <t>2026-07-27T06:03:56.200940</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-27T05:39:29.066959</t>
+          <t>2026-07-27T06:05:08.102136</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-27T00:23:32.727849</t>
+          <t>2026-07-27T06:04:13.294712</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-24T05:21:32.385809</t>
+          <t>2026-07-27T06:00:43.002169</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-27 07:31:20
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -564,7 +564,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-27T06:03:56.200940</t>
+          <t>2026-07-27T07:12:01.492589</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -729,30 +729,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>wcw</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "523629175a3fa50a266a93dd42f72c73eab7a7973bf469fa99484d960dc64dae", "salt": "f18a6bee64d0c036037d4d03cbe4a248051c6973c8b90bbfb565b068c5112c9a", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-21T04:29:08.529075</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2026-07-27T06:05:08.102136</t>
-        </is>
-      </c>
+          <t>2026-07-27T07:31:20.189926</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>否</t>
@@ -767,28 +763,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>xjq-cs</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-27T00:22:56.634377</t>
+          <t>2026-07-21T04:29:08.529075</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-27T06:04:13.294712</t>
+          <t>2026-07-27T06:05:08.102136</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -805,28 +801,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq-cs</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:24.754665</t>
+          <t>2026-07-27T00:22:56.634377</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-24T08:08:35.784199</t>
+          <t>2026-07-27T06:04:13.294712</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -843,12 +839,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>yjl</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -859,12 +855,12 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-21T14:29:59.201564</t>
+          <t>2026-07-21T05:24:24.754665</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-22T07:45:30.020648</t>
+          <t>2026-07-27T06:12:31.801664</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -881,12 +877,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -897,12 +893,12 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
+          <t>2026-07-21T14:29:59.201564</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-23T05:43:14.630942</t>
+          <t>2026-07-22T07:45:30.020648</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -919,36 +915,74 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>2026-07-27T06:00:43.002169</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-27 07:31:58
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -915,30 +915,26 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjx</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "361171e623fc60895ec40f99a6182c27dbb75b5f188cc9ff1a2d3101435abfce", "salt": "9b49c3bf8214dae2038c34380aae01b7c52095684ddbfe01cb6b3f37ee738001", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>2026-07-23T05:43:14.630942</t>
-        </is>
-      </c>
+          <t>2026-07-27T07:31:57.793210</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>否</t>
@@ -953,36 +949,74 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>2026-07-27T06:00:43.002169</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-27 07:32:52
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>bugtest_3439</t>
+          <t>dajinyu</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"hash": "683933ba61b6bf861495d8ae7ca4cf617b20e96a357e17d9f81e6446443adbd1", "salt": "32fd874d74eb06438fd92eb0ec431fa87836ae390370266901c2c7f900ec0432", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "bf8f6de799a7eed9960cc632206baf3714cb8ff2c80be5ed9b4da42cb43f1479", "salt": "7912bbead6671352fdc02410d7dde4006511e2a25d395403478fe021eb682307", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,10 +525,14 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-21T05:36:44.829615</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>2026-07-24T07:40:42.773933</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-07-27T07:12:01.492589</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>否</t>
@@ -543,30 +547,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>dajinyu</t>
+          <t>flora</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"hash": "bf8f6de799a7eed9960cc632206baf3714cb8ff2c80be5ed9b4da42cb43f1479", "salt": "7912bbead6671352fdc02410d7dde4006511e2a25d395403478fe021eb682307", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "5fc51a63f31c86fafce838506de34c1a4822c35e4eb96313622bb3bb12ddb27a", "salt": "046da8c3e3793dc75e716aca13e50e008d0489f7bf9f7dd8e57f0f4b3420154f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-24T07:40:42.773933</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-07-27T07:12:01.492589</t>
-        </is>
-      </c>
+          <t>2026-07-21T05:26:59.748591</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>否</t>
@@ -581,26 +581,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>flora</t>
+          <t>lhl</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "5fc51a63f31c86fafce838506de34c1a4822c35e4eb96313622bb3bb12ddb27a", "salt": "046da8c3e3793dc75e716aca13e50e008d0489f7bf9f7dd8e57f0f4b3420154f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "f8f8de6fab17c4156f58d63b8032586f5475107dd455afb48f34c51ec5863671", "salt": "87e67563dcab6b352e8fb4ae69ea09406ee6ab46bf53767a96d80627edf6f1e0", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-21T05:26:59.748591</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>2026-07-23T05:45:42.431806</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-07-24T02:47:09.177183</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>否</t>
@@ -615,12 +619,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>lhl</t>
+          <t>mwh</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"hash": "f8f8de6fab17c4156f58d63b8032586f5475107dd455afb48f34c51ec5863671", "salt": "87e67563dcab6b352e8fb4ae69ea09406ee6ab46bf53767a96d80627edf6f1e0", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "04849fccab8734257b614a7f3606554f8caeba646c486aa184611893df552b60", "salt": "ecd2366a8275ec9f74a4608b7f239ed77288c66e565865577cd6b899ea48ec90", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -631,12 +635,12 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-23T05:45:42.431806</t>
+          <t>2026-07-23T07:28:50.402064</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-24T02:47:09.177183</t>
+          <t>2026-07-23T11:12:36.939226</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -653,12 +657,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>mwh</t>
+          <t>shj</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"hash": "04849fccab8734257b614a7f3606554f8caeba646c486aa184611893df552b60", "salt": "ecd2366a8275ec9f74a4608b7f239ed77288c66e565865577cd6b899ea48ec90", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "7c63b110a98ad88e9bf4c0a68dcfebf94347e45d54fa8a9860cf55eb3f1d407f", "salt": "335cfcd0dadc5e14e7b562b1c9597812c9c90bbb9f9d57b2872293fc6edbf73a", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -669,14 +673,10 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-23T07:28:50.402064</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2026-07-23T11:12:36.939226</t>
-        </is>
-      </c>
+          <t>2026-07-27T07:32:31.391838</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>否</t>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-27 07:33:47
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -987,12 +987,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>zgq</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "42e9e2fcadb761e5244556575aa4721442bf4729923fe17ff697599fb3bfa3d8", "salt": "83ee0fb089092591226ebbc227dd6d8ba7321553991bb009e39107346ff95b5e", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1003,20 +1003,54 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
+          <t>2026-07-27T07:33:47.301488</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>2026-07-27T06:00:43.002169</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-27 07:34:15
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -763,30 +763,26 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>wyh</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "fd999b2775feceef3dd0d513d427a5e1c3bb5409cf196a95bfdcface07a1e9a4", "salt": "564892c52ed8fbb57ab6590266acae5b165cd6416a3b553db9a65a59d3bd1a4b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-21T04:29:08.529075</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-07-27T06:05:08.102136</t>
-        </is>
-      </c>
+          <t>2026-07-27T07:34:14.901381</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>否</t>
@@ -801,28 +797,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>xjq-cs</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-27T00:22:56.634377</t>
+          <t>2026-07-21T04:29:08.529075</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-27T06:04:13.294712</t>
+          <t>2026-07-27T06:05:08.102136</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -839,28 +835,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq-cs</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:24.754665</t>
+          <t>2026-07-27T00:22:56.634377</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-27T06:12:31.801664</t>
+          <t>2026-07-27T06:04:13.294712</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -877,12 +873,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>yjl</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -893,12 +889,12 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-21T14:29:59.201564</t>
+          <t>2026-07-21T05:24:24.754665</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-22T07:45:30.020648</t>
+          <t>2026-07-27T06:12:31.801664</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -915,26 +911,30 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>yjx</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{"hash": "361171e623fc60895ec40f99a6182c27dbb75b5f188cc9ff1a2d3101435abfce", "salt": "9b49c3bf8214dae2038c34380aae01b7c52095684ddbfe01cb6b3f37ee738001", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-27T07:31:57.793210</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>2026-07-21T14:29:59.201564</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-07-22T07:45:30.020648</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>否</t>
@@ -949,30 +949,26 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjx</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "361171e623fc60895ec40f99a6182c27dbb75b5f188cc9ff1a2d3101435abfce", "salt": "9b49c3bf8214dae2038c34380aae01b7c52095684ddbfe01cb6b3f37ee738001", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>2026-07-23T05:43:14.630942</t>
-        </is>
-      </c>
+          <t>2026-07-27T07:31:57.793210</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>否</t>
@@ -987,26 +983,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>zgq</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>{"hash": "42e9e2fcadb761e5244556575aa4721442bf4729923fe17ff697599fb3bfa3d8", "salt": "83ee0fb089092591226ebbc227dd6d8ba7321553991bb009e39107346ff95b5e", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-27T07:33:47.301488</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>否</t>
@@ -1021,12 +1021,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>zgq</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "42e9e2fcadb761e5244556575aa4721442bf4729923fe17ff697599fb3bfa3d8", "salt": "83ee0fb089092591226ebbc227dd6d8ba7321553991bb009e39107346ff95b5e", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1037,20 +1037,54 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
+          <t>2026-07-27T07:33:47.301488</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>2026-07-27T06:00:43.002169</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-27 08:54:23
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -768,7 +768,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "fd999b2775feceef3dd0d513d427a5e1c3bb5409cf196a95bfdcface07a1e9a4", "salt": "564892c52ed8fbb57ab6590266acae5b165cd6416a3b553db9a65a59d3bd1a4b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "7e376ec0f7cf89589117757ec6dfb9cdb10bc4f0f3af2cb841264f83ada223cf", "salt": "0804bee696543f754b89985bab99c738c7fb5c319f324d87fa95e6f443e6ea2b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-27T06:05:08.102136</t>
+          <t>2026-07-27T08:37:03.192902</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq归档项目 - 2026-07-28 01:31:03
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -782,7 +782,11 @@
           <t>2026-07-27T07:34:14.901381</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-07-27T08:54:37.787742</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>否</t>
@@ -818,7 +822,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-27T08:37:03.192902</t>
+          <t>2026-07-28T01:29:48.184623</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq编辑项目 - 2026-07-28 07:34:25
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -748,7 +748,11 @@
           <t>2026-07-27T07:31:20.189926</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-07-28T03:03:51.787126</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>否</t>
@@ -784,7 +788,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-27T08:54:37.787742</t>
+          <t>2026-07-28T01:31:45.481348</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1044,7 +1048,11 @@
           <t>2026-07-27T07:33:47.301488</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-07-28T07:06:56.684466</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
           <t>否</t>

</xml_diff>

<commit_message>
[API同步] ycx编辑项目 - 2026-07-29 00:58:43
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-27T07:12:01.492589</t>
+          <t>2026-07-28T12:10:07.684273</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -676,7 +676,11 @@
           <t>2026-07-27T07:32:31.391838</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-07-28T08:34:11.679682</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>否</t>
@@ -826,7 +830,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-28T01:29:48.184623</t>
+          <t>2026-07-29T00:56:30.985306</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -902,7 +906,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-27T06:12:31.801664</t>
+          <t>2026-07-29T00:57:45.885619</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -976,7 +980,11 @@
           <t>2026-07-27T07:31:57.793210</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-07-28T08:49:19.781897</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>否</t>

</xml_diff>

<commit_message>
[API同步] xjq编辑项目 - 2026-07-29 01:33:39
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-28T08:34:11.679682</t>
+          <t>2026-07-29T01:29:25.791538</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-28T01:31:45.481348</t>
+          <t>2026-07-29T01:24:42.590805</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-28T07:06:56.684466</t>
+          <t>2026-07-29T01:29:12.890535</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-27T06:00:43.002169</t>
+          <t>2026-07-29T01:28:09.988552</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] tjs新增项目: 蓝牙工装 - 2026-07-30 08:32:03
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-29T11:45:46.189853</t>
+          <t>2026-07-30T08:10:36.180254</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-29T01:45:25.180445</t>
+          <t>2026-07-30T08:31:07.183401</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-30T05:17:43.583399</t>
+          <t>2026-07-30T07:52:49.586345</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-30T00:24:16.387078</t>
+          <t>2026-07-30T07:32:52.886079</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-30T00:44:46.290266</t>
+          <t>2026-07-30T07:56:05.888332</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-31 11:41:57
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -750,7 +750,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-31T11:20:51.834486</t>
+          <t>2026-07-31T11:39:16.210498</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"hash": "93b93541a317533e413a8971c0372e6485844b55c06691e703267f2718323e8f", "salt": "0e0bb8a301b157df497cdd4e44fd5dd42b50bf91cc69b8114d9662b960698d77", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9892de7861e71a41cb93a48d7c5ba7fd627c2784aade8191566cf9a13c222d8a", "salt": "44b594e538222ebf7f9ab52c2b297487711cc67af5b37d6058b2d9dfc44221ef", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-24T08:08:35.784199</t>
+          <t>2026-07-31T11:40:45.000972</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-31 11:46:21
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -826,7 +826,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-31T11:40:45.000972</t>
+          <t>2026-07-31T11:42:10.503687</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -919,12 +919,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>zgj</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "0e5b6b8ce4489ad48ac71ce0792939a00dd66859b1fdab50c596e30a087b475b", "salt": "a6a0196dc816a9955239ef176848211c949eb20e49ae0ff8577524cae63e50af", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -935,20 +935,54 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
+          <t>2026-07-31T11:46:20.507021</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>2026-07-24T05:21:32.385809</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-31 11:46:42
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -729,30 +729,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>wyh</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "88b518183bbf2a902c1e8e1388398b0730dc6aad355ed5056e9879f1381e09e1", "salt": "544a3103ff54ee895ae3021ce15f20c0d901967ab39a87b4891430dd9be5f822", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-21T04:29:08.529075</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2026-07-31T11:39:16.210498</t>
-        </is>
-      </c>
+          <t>2026-07-31T11:46:41.613282</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>否</t>
@@ -767,28 +763,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>xjq-cs</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-27T00:22:56.634377</t>
+          <t>2026-07-21T04:29:08.529075</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-27T00:23:32.727849</t>
+          <t>2026-07-31T11:39:16.210498</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -805,28 +801,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq-cs</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"hash": "9892de7861e71a41cb93a48d7c5ba7fd627c2784aade8191566cf9a13c222d8a", "salt": "44b594e538222ebf7f9ab52c2b297487711cc67af5b37d6058b2d9dfc44221ef", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:24.754665</t>
+          <t>2026-07-27T00:22:56.634377</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-31T11:42:10.503687</t>
+          <t>2026-07-27T00:23:32.727849</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -843,12 +839,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>yjl</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9892de7861e71a41cb93a48d7c5ba7fd627c2784aade8191566cf9a13c222d8a", "salt": "44b594e538222ebf7f9ab52c2b297487711cc67af5b37d6058b2d9dfc44221ef", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -859,12 +855,12 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-21T14:29:59.201564</t>
+          <t>2026-07-21T05:24:24.754665</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-22T07:45:30.020648</t>
+          <t>2026-07-31T11:42:10.503687</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -881,12 +877,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -897,12 +893,12 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
+          <t>2026-07-21T14:29:59.201564</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-23T05:43:14.630942</t>
+          <t>2026-07-22T07:45:30.020648</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -919,26 +915,30 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>zgj</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{"hash": "0e5b6b8ce4489ad48ac71ce0792939a00dd66859b1fdab50c596e30a087b475b", "salt": "a6a0196dc816a9955239ef176848211c949eb20e49ae0ff8577524cae63e50af", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-31T11:46:20.507021</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>否</t>
@@ -953,12 +953,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>zgj</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "0e5b6b8ce4489ad48ac71ce0792939a00dd66859b1fdab50c596e30a087b475b", "salt": "a6a0196dc816a9955239ef176848211c949eb20e49ae0ff8577524cae63e50af", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -969,20 +969,54 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
+          <t>2026-07-31T11:46:20.507021</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>2026-07-24T05:21:32.385809</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-31 11:47:00
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -691,30 +691,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tjs</t>
+          <t>shj</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "ff481015559bcbcaf62f8a10eb4476b76b9a48030e189473eae593876bc87d59", "salt": "e95f6a23a1483d8bdc1dfc159589dd1a1232bb5529eb7da8c629950f6aa68f46", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "d8848c80c2ba51e092d3eafbb5c6aef9713cf01c29779b5fe664f83e85248e46", "salt": "671c5c48a46d4faa6224071587573c74eec60b4efd9eebde234109c41c2d92a7", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-23T07:16:34.409165</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2026-07-24T05:51:30.972507</t>
-        </is>
-      </c>
+          <t>2026-07-31T11:47:00.205006</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>否</t>
@@ -729,26 +725,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>wyh</t>
+          <t>tjs</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"hash": "88b518183bbf2a902c1e8e1388398b0730dc6aad355ed5056e9879f1381e09e1", "salt": "544a3103ff54ee895ae3021ce15f20c0d901967ab39a87b4891430dd9be5f822", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "ff481015559bcbcaf62f8a10eb4476b76b9a48030e189473eae593876bc87d59", "salt": "e95f6a23a1483d8bdc1dfc159589dd1a1232bb5529eb7da8c629950f6aa68f46", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-31T11:46:41.613282</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>2026-07-23T07:16:34.409165</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-07-24T05:51:30.972507</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>否</t>
@@ -763,30 +763,26 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>wyh</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "88b518183bbf2a902c1e8e1388398b0730dc6aad355ed5056e9879f1381e09e1", "salt": "544a3103ff54ee895ae3021ce15f20c0d901967ab39a87b4891430dd9be5f822", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-21T04:29:08.529075</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-07-31T11:39:16.210498</t>
-        </is>
-      </c>
+          <t>2026-07-31T11:46:41.613282</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>否</t>
@@ -801,28 +797,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>xjq-cs</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-27T00:22:56.634377</t>
+          <t>2026-07-21T04:29:08.529075</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-27T00:23:32.727849</t>
+          <t>2026-07-31T11:39:16.210498</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -839,28 +835,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq-cs</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"hash": "9892de7861e71a41cb93a48d7c5ba7fd627c2784aade8191566cf9a13c222d8a", "salt": "44b594e538222ebf7f9ab52c2b297487711cc67af5b37d6058b2d9dfc44221ef", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:24.754665</t>
+          <t>2026-07-27T00:22:56.634377</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-31T11:42:10.503687</t>
+          <t>2026-07-27T00:23:32.727849</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -877,12 +873,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>yjl</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9892de7861e71a41cb93a48d7c5ba7fd627c2784aade8191566cf9a13c222d8a", "salt": "44b594e538222ebf7f9ab52c2b297487711cc67af5b37d6058b2d9dfc44221ef", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -893,12 +889,12 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-21T14:29:59.201564</t>
+          <t>2026-07-21T05:24:24.754665</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-22T07:45:30.020648</t>
+          <t>2026-07-31T11:42:10.503687</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -915,12 +911,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -931,12 +927,12 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
+          <t>2026-07-21T14:29:59.201564</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-23T05:43:14.630942</t>
+          <t>2026-07-22T07:45:30.020648</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -953,26 +949,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>zgj</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{"hash": "0e5b6b8ce4489ad48ac71ce0792939a00dd66859b1fdab50c596e30a087b475b", "salt": "a6a0196dc816a9955239ef176848211c949eb20e49ae0ff8577524cae63e50af", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-31T11:46:20.507021</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>否</t>
@@ -987,12 +987,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>zgj</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "0e5b6b8ce4489ad48ac71ce0792939a00dd66859b1fdab50c596e30a087b475b", "salt": "a6a0196dc816a9955239ef176848211c949eb20e49ae0ff8577524cae63e50af", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1003,20 +1003,54 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
+          <t>2026-07-31T11:46:20.507021</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>2026-07-24T05:21:32.385809</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-07-31 11:47:22
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -949,30 +949,26 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjx</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "670f48cc94dacd174f598704f7809f8d64413ccfdee3479ca506a5d022785533", "salt": "5932a668fac8f2e7183150418c4969646cc83c0ab793127c78b0932a86ba8abb", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>2026-07-23T05:43:14.630942</t>
-        </is>
-      </c>
+          <t>2026-07-31T11:47:21.704683</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>否</t>
@@ -987,26 +983,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>zgj</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>{"hash": "0e5b6b8ce4489ad48ac71ce0792939a00dd66859b1fdab50c596e30a087b475b", "salt": "a6a0196dc816a9955239ef176848211c949eb20e49ae0ff8577524cae63e50af", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-31T11:46:20.507021</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>否</t>
@@ -1021,12 +1021,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>zgj</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "0e5b6b8ce4489ad48ac71ce0792939a00dd66859b1fdab50c596e30a087b475b", "salt": "a6a0196dc816a9955239ef176848211c949eb20e49ae0ff8577524cae63e50af", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1037,20 +1037,54 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
+          <t>2026-07-31T11:46:20.507021</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>2026-07-24T05:21:32.385809</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 用户xjq增量同步，重试推送 - 2026-08-03 01:03:19
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-24T12:42:40.776957</t>
+          <t>2026-08-03T00:32:14.513108</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-23T11:12:36.939226</t>
+          <t>2026-08-01T03:22:24.904953</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-31T11:39:16.210498</t>
+          <t>2026-08-03T01:02:39.904191</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-08-03 01:14:48
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -763,12 +763,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>wyh</t>
+          <t>wcw</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"hash": "88b518183bbf2a902c1e8e1388398b0730dc6aad355ed5056e9879f1381e09e1", "salt": "544a3103ff54ee895ae3021ce15f20c0d901967ab39a87b4891430dd9be5f822", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6f530e3022e1807247343dee042a126c1d1db3d1701cfbf0c635b5089ebea71c", "salt": "3368f337f813c596cbfafbd1bc2ffb53d119020a778a424e1df6f8d37d82d2a6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -779,7 +779,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-31T11:46:41.613282</t>
+          <t>2026-08-03T01:14:48.004063</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -797,30 +797,26 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>xjq</t>
+          <t>wyh</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "88b518183bbf2a902c1e8e1388398b0730dc6aad355ed5056e9879f1381e09e1", "salt": "544a3103ff54ee895ae3021ce15f20c0d901967ab39a87b4891430dd9be5f822", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-21T04:29:08.529075</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2026-08-03T01:02:39.904191</t>
-        </is>
-      </c>
+          <t>2026-07-31T11:46:41.613282</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>否</t>
@@ -835,28 +831,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>xjq-cs</t>
+          <t>xjq</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "e2b4750a7223681a0b94867c4f7cde9c57571a6ea9453158a19f1d0236e5cbfc", "salt": "55b207a6f3ae59afd188365748815a49df0393de7e85c1750f4c2f996dfbf812", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-27T00:22:56.634377</t>
+          <t>2026-07-21T04:29:08.529075</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-27T00:23:32.727849</t>
+          <t>2026-08-03T01:02:39.904191</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -873,28 +869,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ycx</t>
+          <t>xjq-cs</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{"hash": "9892de7861e71a41cb93a48d7c5ba7fd627c2784aade8191566cf9a13c222d8a", "salt": "44b594e538222ebf7f9ab52c2b297487711cc67af5b37d6058b2d9dfc44221ef", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "34e9d58e9de5168d2e3eb08800b42833d49b5809fda00245684042f4a7baf291", "salt": "486ff56eb2d75943a225e176eb30d5046ef2990a29011a3115791dc7868c8da6", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:24.754665</t>
+          <t>2026-07-27T00:22:56.634377</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-31T11:42:10.503687</t>
+          <t>2026-07-27T00:23:32.727849</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -911,12 +907,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>yjl</t>
+          <t>ycx</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "9892de7861e71a41cb93a48d7c5ba7fd627c2784aade8191566cf9a13c222d8a", "salt": "44b594e538222ebf7f9ab52c2b297487711cc67af5b37d6058b2d9dfc44221ef", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -927,12 +923,12 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-21T14:29:59.201564</t>
+          <t>2026-07-21T05:24:24.754665</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-22T07:45:30.020648</t>
+          <t>2026-08-03T01:12:17.016417</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -949,26 +945,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>yjx</t>
+          <t>yjl</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{"hash": "670f48cc94dacd174f598704f7809f8d64413ccfdee3479ca506a5d022785533", "salt": "5932a668fac8f2e7183150418c4969646cc83c0ab793127c78b0932a86ba8abb", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "994b7926900770e173c7eddf88293355ddcfb7b8ac12b649ae4864bbe0662b52", "salt": "cb15b293dff2f3bc9a3bc84589045aaaa53f4cc09a48b27ad0c8866ebff2bb27", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-31T11:47:21.704683</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>2026-07-21T14:29:59.201564</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-07-22T07:45:30.020648</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>否</t>
@@ -983,30 +983,26 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>yzz</t>
+          <t>yjx</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "670f48cc94dacd174f598704f7809f8d64413ccfdee3479ca506a5d022785533", "salt": "5932a668fac8f2e7183150418c4969646cc83c0ab793127c78b0932a86ba8abb", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-21T05:24:08.554209</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>2026-07-23T05:43:14.630942</t>
-        </is>
-      </c>
+          <t>2026-07-31T11:47:21.704683</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>否</t>
@@ -1021,26 +1017,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>zgj</t>
+          <t>yzz</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>{"hash": "0e5b6b8ce4489ad48ac71ce0792939a00dd66859b1fdab50c596e30a087b475b", "salt": "a6a0196dc816a9955239ef176848211c949eb20e49ae0ff8577524cae63e50af", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>editor</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-31T11:46:20.507021</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+          <t>2026-07-21T05:24:08.554209</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-07-23T05:43:14.630942</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
           <t>否</t>
@@ -1055,12 +1055,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>zgj</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "0e5b6b8ce4489ad48ac71ce0792939a00dd66859b1fdab50c596e30a087b475b", "salt": "a6a0196dc816a9955239ef176848211c949eb20e49ae0ff8577524cae63e50af", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1071,20 +1071,54 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
+          <t>2026-07-31T11:46:20.507021</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>2026-07-24T05:21:32.385809</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-08-03 01:59:00
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -696,7 +696,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"hash": "d8848c80c2ba51e092d3eafbb5c6aef9713cf01c29779b5fe664f83e85248e46", "salt": "671c5c48a46d4faa6224071587573c74eec60b4efd9eebde234109c41c2d92a7", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "671a0ff23792391c26f04884ea854f41438efbbcf2c8220ad1d0c9c82fb2ac33", "salt": "0fec9f40521e1f9db12d61c3462be0ba98fcb0db7b80bd2c9d5e0206f0c616aa", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -710,7 +710,11 @@
           <t>2026-07-31T11:47:00.205006</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-08-03T01:57:54.992246</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>否</t>
@@ -1089,12 +1093,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>zky</t>
+          <t>zgq</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6d7e9354db1e8eb8462c606a7b473ab1a0e986ba1759d44680923e1a7083b289", "salt": "ef71db02213b66b058153126fbfda3c7ea30b85e161321504589c2760983690b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1105,20 +1109,54 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
+          <t>2026-08-03T01:58:59.390504</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>zky</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
           <t>2026-07-23T00:58:22.865573</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>2026-07-24T05:21:32.385809</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-08-03 01:59:08
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1059,12 +1059,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>zgj</t>
+          <t>zgq</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>{"hash": "0e5b6b8ce4489ad48ac71ce0792939a00dd66859b1fdab50c596e30a087b475b", "salt": "a6a0196dc816a9955239ef176848211c949eb20e49ae0ff8577524cae63e50af", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "6d7e9354db1e8eb8462c606a7b473ab1a0e986ba1759d44680923e1a7083b289", "salt": "ef71db02213b66b058153126fbfda3c7ea30b85e161321504589c2760983690b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1075,7 +1075,7 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-31T11:46:20.507021</t>
+          <t>2026-08-03T01:58:59.390504</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1093,12 +1093,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>zgq</t>
+          <t>zky</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>{"hash": "6d7e9354db1e8eb8462c606a7b473ab1a0e986ba1759d44680923e1a7083b289", "salt": "ef71db02213b66b058153126fbfda3c7ea30b85e161321504589c2760983690b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1109,54 +1109,20 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-03T01:58:59.390504</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
+          <t>2026-07-23T00:58:22.865573</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-07-24T05:21:32.385809</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>zky</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>{"hash": "22f101ce7faa14d6655bc466c29d8d904b8be747684fc45120da0e8a27ed09ac", "salt": "dcdc4612d3bab2cdc8c9675342ece56641419f98dbf7a11da3fa8fd4c6afc20b", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2026-07-23T00:58:22.865573</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>2026-07-24T05:21:32.385809</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
[API同步] xjq编辑项目 - 2026-08-03 02:20:31
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -786,7 +786,11 @@
           <t>2026-08-03T01:14:48.004063</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-08-03T02:15:16.184474</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>否</t>
@@ -856,7 +860,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-03T01:51:51.787264</t>
+          <t>2026-08-03T02:16:10.985374</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -970,7 +974,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-07-22T07:45:30.020648</t>
+          <t>2026-08-03T02:05:20.789897</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1078,7 +1082,11 @@
           <t>2026-08-03T01:58:59.390504</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-08-03T01:59:31.685125</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>否</t>
@@ -1114,7 +1122,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-24T05:21:32.385809</t>
+          <t>2026-08-03T02:07:18.896654</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq拒绝审批ROW-150 - 2026-08-03 08:51:38
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-03T00:32:14.513108</t>
+          <t>2026-08-03T02:29:35.588699</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-01T03:22:24.904953</t>
+          <t>2026-08-03T03:04:10.891574</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-24T05:51:30.972507</t>
+          <t>2026-08-03T02:28:18.497591</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-03T02:16:10.985374</t>
+          <t>2026-08-03T07:04:42.514317</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-03T02:05:20.789897</t>
+          <t>2026-08-03T07:06:06.219818</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1030,12 +1030,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>{"hash": "3949644cf105795011c36c45878c02dfd130d2cfd4140aa595abc5d4feb1a2fd", "salt": "c771b7150781800012258cf10193ad2678f305e13c6bf479aa00f46f8b4a7191", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "a14429cd3d840b5204a0e8b15e00406c8bf4e887613fbe4d107dac0b746aeffb", "salt": "a1c87807f27d480d3f9f7476ebc6c48149061659d85d5cfa22525f183a3999a0", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-23T05:43:14.630942</t>
+          <t>2026-08-03T07:08:06.809526</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq编辑项目 - 2026-08-04 00:49:58
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -860,7 +860,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-03T07:04:42.514317</t>
+          <t>2026-08-04T00:49:08.107981</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-03T01:59:31.685125</t>
+          <t>2026-08-03T11:12:25.219104</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-03T02:07:18.896654</t>
+          <t>2026-08-04T00:31:39.507317</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-08-04 02:29:34
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -936,7 +936,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-03T01:12:17.016417</t>
+          <t>2026-08-04T01:10:35.811231</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] 更新用户数据 - 2026-08-04 02:30:18
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -586,12 +586,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"hash": "5fc51a63f31c86fafce838506de34c1a4822c35e4eb96313622bb3bb12ddb27a", "salt": "046da8c3e3793dc75e716aca13e50e008d0489f7bf9f7dd8e57f0f4b3420154f", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
+          <t>{"hash": "16627e8ee3a59f61a252e5f8d1c9946c2a88119682e6ca10bf4b72f9da00e7b6", "salt": "492efd53dd2da5a09edb009233717a19e257c0c697db16f714925ee7cd46d531", "iterations": 200000, "algorithm": "PBKDF2-HMAC-SHA256"}</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>

</xml_diff>

<commit_message>
[API同步] 用户flora增量同步，重试推送 - 2026-08-04 08:16:48
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -600,7 +600,11 @@
           <t>2026-07-21T05:26:59.748591</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-08-04T08:12:19.216937</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>否</t>

</xml_diff>

<commit_message>
[API同步] ycx编辑项目 - 2026-08-05 00:35:41
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-03T02:29:35.588699</t>
+          <t>2026-08-04T09:22:47.811579</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-08-03T02:15:16.184474</t>
+          <t>2026-08-04T08:18:42.017862</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-04T01:10:35.811231</t>
+          <t>2026-08-05T00:35:00.319709</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] zgq撤回审批OP-20260804-002 - 2026-08-05 06:21:28
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-08-04T08:12:19.216937</t>
+          <t>2026-08-05T03:21:04.120630</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-08-04T08:18:42.017862</t>
+          <t>2026-08-05T03:01:13.816984</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-03T11:12:25.219104</t>
+          <t>2026-08-05T02:08:38.814491</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">

</xml_diff>

<commit_message>
[API同步] xjq拒绝审批OP-20260805-001 - 2026-08-05 08:33:22
</commit_message>
<xml_diff>
--- a/用户管理.xlsx
+++ b/用户管理.xlsx
@@ -864,7 +864,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-04T00:49:08.107981</t>
+          <t>2026-08-05T08:32:42.614004</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-04T00:31:39.507317</t>
+          <t>2026-08-05T08:32:57.508978</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">

</xml_diff>